<commit_message>
Finalized with reports List of contracts and Cashflow calendar along with the report options Base and Base plus Addendum
</commit_message>
<xml_diff>
--- a/src/main/resources/ru/stnovator/finassist/report/cashflow-calendar.xlsx
+++ b/src/main/resources/ru/stnovator/finassist/report/cashflow-calendar.xlsx
@@ -11,19 +11,19 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" name="Header" vbProcedure="false">Sheet1!$A$1:$T$2</definedName>
-    <definedName function="false" hidden="false" name="Calendar_header" vbProcedure="false">Sheet1!$A$4:$H$4</definedName>
-    <definedName function="false" hidden="false" name="Calendar_dynamic_header" vbProcedure="false">Sheet1!$I$4</definedName>
-    <definedName function="false" hidden="false" name="Calendar_master_data" vbProcedure="false">Sheet1!$A$5:$H$5</definedName>
-    <definedName function="false" hidden="false" name="Calendar" vbProcedure="false">Sheet1!$I$5</definedName>
-    <definedName function="false" hidden="false" name="CalendarTotals" vbProcedure="false">Sheet1!$A$7:$T$7</definedName>
+    <definedName function="false" hidden="false" name="Header" vbProcedure="false">Sheet1!$A$1:$V$2</definedName>
+    <definedName function="false" hidden="false" name="Calendar_header" vbProcedure="false">Sheet1!$A$4:$J$4</definedName>
+    <definedName function="false" hidden="false" name="Calendar_dynamic_header" vbProcedure="false">Sheet1!$K$4</definedName>
+    <definedName function="false" hidden="false" name="Calendar_master_data" vbProcedure="false">Sheet1!$A$5:$J$5</definedName>
+    <definedName function="false" hidden="false" name="Calendar" vbProcedure="false">Sheet1!$K$5</definedName>
+    <definedName function="false" hidden="false" name="CalendarTotals" vbProcedure="false">Sheet1!$A$7:$V$7</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
   <si>
     <t xml:space="preserve">${title}</t>
   </si>
@@ -46,6 +46,12 @@
     <t xml:space="preserve">Показатель</t>
   </si>
   <si>
+    <t xml:space="preserve">Источник плана</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Доп. соглашение</t>
+  </si>
+  <si>
     <t xml:space="preserve">План контракта</t>
   </si>
   <si>
@@ -71,6 +77,12 @@
   </si>
   <si>
     <t xml:space="preserve">${measureName}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">${planSource}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">${addendumInfo}</t>
   </si>
   <si>
     <t xml:space="preserve">${contractPlannedSum}</t>
@@ -532,18 +544,20 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:T7"/>
+  <dimension ref="A1:V7"/>
   <sheetFormatPr defaultColWidth="12" defaultRowHeight="18" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="18" style="0" hidden="false" customWidth="true" outlineLevel="0" collapsed="false"/>
     <col min="2" max="2" width="22" style="0" hidden="false" customWidth="true" outlineLevel="0" collapsed="false"/>
     <col min="3" max="3" width="34" style="0" hidden="false" customWidth="true" outlineLevel="0" collapsed="false"/>
     <col min="4" max="4" width="17" style="0" hidden="false" customWidth="true" outlineLevel="0" collapsed="false"/>
-    <col min="5" max="5" width="14" style="0" hidden="false" customWidth="true" outlineLevel="0" collapsed="false"/>
-    <col min="6" max="6" width="11.5" style="0" hidden="false" customWidth="true" outlineLevel="0" collapsed="false"/>
-    <col min="7" max="7" width="11.5" style="0" hidden="false" customWidth="true" outlineLevel="0" collapsed="false"/>
-    <col min="8" max="8" width="14" style="0" hidden="false" customWidth="true" outlineLevel="0" collapsed="false"/>
-    <col min="9" max="20" width="11.5" style="0" hidden="false" customWidth="true" outlineLevel="0" collapsed="false"/>
+    <col min="5" max="5" width="16" style="0" hidden="false" customWidth="true" outlineLevel="0" collapsed="false"/>
+    <col min="6" max="6" width="22" style="0" hidden="false" customWidth="true" outlineLevel="0" collapsed="false"/>
+    <col min="7" max="7" width="14" style="0" hidden="false" customWidth="true" outlineLevel="0" collapsed="false"/>
+    <col min="8" max="8" width="11.5" style="0" hidden="false" customWidth="true" outlineLevel="0" collapsed="false"/>
+    <col min="9" max="9" width="11.5" style="0" hidden="false" customWidth="true" outlineLevel="0" collapsed="false"/>
+    <col min="10" max="10" width="14" style="0" hidden="false" customWidth="true" outlineLevel="0" collapsed="false"/>
+    <col min="11" max="22" width="11.5" style="0" hidden="false" customWidth="true" outlineLevel="0" collapsed="false"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="true">
@@ -569,6 +583,8 @@
       <c r="R1" s="1"/>
       <c r="S1" s="1"/>
       <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="1"/>
     </row>
     <row r="2" ht="22" customHeight="true">
       <c r="A2" s="2" t="s">
@@ -595,6 +611,8 @@
       <c r="R2" s="10"/>
       <c r="S2" s="10"/>
       <c r="T2" s="10"/>
+      <c r="U2" s="10"/>
+      <c r="V2" s="10"/>
     </row>
     <row r="3" ht="10" customHeight="true">
       <c r="A3"/>
@@ -617,6 +635,8 @@
       <c r="R3"/>
       <c r="S3"/>
       <c r="T3"/>
+      <c r="U3"/>
+      <c r="V3"/>
     </row>
     <row r="4" ht="32" customHeight="true">
       <c r="A4" s="6" t="s">
@@ -631,49 +651,61 @@
       <c r="D4" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="6" t="s">
         <v>8</v>
       </c>
       <c r="G4" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="H4" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="H4" s="8" t="s">
+      <c r="I4" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K4" s="6" t="s">
         <v>11</v>
-      </c>
-      <c r="I4" s="6" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="5" ht="28" customHeight="true">
       <c r="A5" s="3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E5" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="F5" s="9" t="s">
         <v>17</v>
       </c>
+      <c r="E5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="G5" s="9" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>18</v>
+        <v>21</v>
+      </c>
+      <c r="I5" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="J5" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="6" ht="10" customHeight="true">
@@ -697,72 +729,80 @@
       <c r="R6"/>
       <c r="S6"/>
       <c r="T6"/>
+      <c r="U6"/>
+      <c r="V6"/>
     </row>
     <row r="7" ht="28" customHeight="true">
       <c r="A7" s="8" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="F7" s="9" t="s">
         <v>17</v>
       </c>
+      <c r="E7" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>25</v>
+      </c>
       <c r="G7" s="9" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J7" s="9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K7" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="L7" s="9" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M7" s="9" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="N7" s="9" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="O7" s="9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="P7" s="9" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="Q7" s="9" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="R7" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="S7" s="9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="T7" s="9" t="s">
-        <v>33</v>
+        <v>35</v>
+      </c>
+      <c r="U7" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="V7" s="9" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:T1"/>
+    <mergeCell ref="A1:V1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.45" right="0.45" top="0.55" bottom="0.55" header="0.3" footer="0.3"/>

</xml_diff>